<commit_message>
Level scaling and stats are now being applied properly when a character levels up. We also scale properly when we gain multiple levels.
</commit_message>
<xml_diff>
--- a/resources/data-imports/Monsters/raid-bosses.xlsx
+++ b/resources/data-imports/Monsters/raid-bosses.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="64">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -200,9 +200,6 @@
   </si>
   <si>
     <t xml:space="preserve">Jester of Time</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delusinal</t>
   </si>
   <si>
     <t xml:space="preserve">Delusional Memories</t>
@@ -224,7 +221,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -245,18 +242,6 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="6.4"/>
-      <color rgb="FF2E3436"/>
-      <name val="Adwaita Sans"/>
       <family val="0"/>
     </font>
   </fonts>
@@ -302,7 +287,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -311,11 +296,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -328,66 +309,6 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF2E3436"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -1204,8 +1125,8 @@
       <c r="H5" s="1" t="n">
         <v>100000000000</v>
       </c>
-      <c r="I5" s="3" t="s">
-        <v>60</v>
+      <c r="I5" s="1" t="n">
+        <v>100000000000</v>
       </c>
       <c r="J5" s="1" t="n">
         <v>4000000000</v>
@@ -1295,7 +1216,7 @@
         <v>0</v>
       </c>
       <c r="AO5" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AQ5" s="1" t="n">
         <v>0.275</v>
@@ -1321,7 +1242,7 @@
         <v>517</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C6" s="1" t="n">
         <v>100000000000</v>
@@ -1432,7 +1353,7 @@
         <v>0</v>
       </c>
       <c r="AO6" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AQ6" s="1" t="n">
         <v>0.275</v>
@@ -1455,7 +1376,7 @@
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C7" s="1" t="n">
         <v>100000000000</v>
@@ -1566,7 +1487,7 @@
         <v>0</v>
       </c>
       <c r="AO7" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AQ7" s="1" t="n">
         <v>0.6</v>

</xml_diff>